<commit_message>
refactor: improve schedule timer system with task-based execution
- Refactor schedule timer to use next execution time tracking instead of last execution
- Add logic thread switching for Lua script execution
- Add func field to schedule model for Lua function name specification
- Add schedule initialization method to calculate initial execution times
- Add next_execution calculation method to schedule model
- Unify schedule script format with function-based execution
- Remove old test scripts (once.lua, repeat.lua)
- Add new unified schedule script implementation
</commit_message>
<xml_diff>
--- a/resources/table/schedule.xlsx
+++ b/resources/table/schedule.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{134F0C37-57D9-4C7E-9333-3901CE85A6A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A15D7F-DDE8-4E69-BDEF-5076983C5359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
   </bookViews>
   <sheets>
     <sheet name="schedule" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -43,22 +43,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>2026-01-23 00:00:00 ~ 2026-01-24 00:00:00</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>repeat</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>0.00:00:30</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026-01-24 00:00:00 ~ 2026-01-24 00:00:00</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>script</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -67,19 +55,39 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>scripts/schedule/repeat.lua</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>scripts/schedule/once.lua</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>TimeSpan?</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>DateRange</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.00:00:10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-01-23 00:00:00 ~ 2026-01-25 00:00:00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>func</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ON_SCHEDULE_0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ON_SCHEDULE_1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scripts/schedule/schedule.lua</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-01-24 01:10:00</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -134,7 +142,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -144,9 +152,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -162,7 +176,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -458,17 +472,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE8D9647-70DB-4352-ABD3-4D2F60838B15}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" style="1"/>
     <col min="4" max="4" width="22.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="1"/>
+    <col min="5" max="5" width="14.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -476,27 +491,33 @@
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>8</v>
+      <c r="E1" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -509,33 +530,42 @@
       <c r="D3" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="E3" s="1" t="s">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" ht="27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="27" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>0</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>7</v>
+      <c r="B5" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
script: Lua script implementation for NPC, mob, and item
- Implement and update NPC, mob, and item Lua scripts
- Add init.lua and CONVERSION_VIOLATIONS.md
- Expand interaction.lua and command.lua
- Remove achievement/quest tables and related C++/model code for script support
- Update dialog, character, mob, server builtins and protocol; HTTP/DB and internal config
</commit_message>
<xml_diff>
--- a/resources/table/schedule.xlsx
+++ b/resources/table/schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A15D7F-DDE8-4E69-BDEF-5076983C5359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E303774C-D7D2-4C8A-9998-6A0CCD3DA840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -88,6 +88,18 @@
   </si>
   <si>
     <t>2026-01-24 01:10:00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1.00:00:00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ON_SCHEDULE_2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1900-01-01 18:00:00</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -566,7 +578,21 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="2"/>
+      <c r="A6" s="1">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
feat: schedule, scripts, lua and table updates
- Update lua.cpp, chat handler, portrait, object_show, worker.script
- Extend command.lua, init.lua, interaction.lua, schedule.lua, server.lua
- Update NPC script and resources (map.xlsx, schedule.xlsx)
</commit_message>
<xml_diff>
--- a/resources/table/schedule.xlsx
+++ b/resources/table/schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E303774C-D7D2-4C8A-9998-6A0CCD3DA840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF311F64-EDE0-4613-BBF8-12B9C117CF52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -100,6 +100,18 @@
   </si>
   <si>
     <t>1900-01-01 18:00:00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1900-01-01 00:00:00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.01:00:00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ON_SCHEDULE_3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -484,7 +496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE8D9647-70DB-4352-ABD3-4D2F60838B15}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.375" style="1" bestFit="1" customWidth="1"/>
@@ -594,8 +606,26 @@
         <v>17</v>
       </c>
     </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>